<commit_message>
Tshirt Addition - 170726
</commit_message>
<xml_diff>
--- a/Mrp.xlsx
+++ b/Mrp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benedictjohn/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benedictjohn/Desktop/JavaScript-course/Asha Books Wholesale Website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE8988C-6010-7442-891A-74B9145090A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1894820-71FD-A840-A4C8-83AE23C7F713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="740" windowWidth="12960" windowHeight="15920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update - 25K minimum
</commit_message>
<xml_diff>
--- a/Mrp.xlsx
+++ b/Mrp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benedictjohn/Desktop/JavaScript-course/Asha Books Wholesale Website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30DC90C4-154C-274C-B5D6-555BB42F6C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10E8192-1F8D-C140-89CB-B4471F5F67BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2282,10 +2282,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J626"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="72.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
@@ -2355,7 +2355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>9780310080008</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>9780310088417</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>9780310090335</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>9780310094067</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>9780310094487</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>9780310158882</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9780310158905</v>
       </c>
@@ -2611,7 +2611,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9780310429401</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>9780310436867</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>9780310441595</v>
       </c>
@@ -2835,7 +2835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>9780310444053</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>9780310445890</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>9780310445906</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>9780310446361</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>9780310446378</v>
       </c>
@@ -3027,7 +3027,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>9780310446422</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>9780310446699</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>9780310446774</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>9780310446828</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>9780310446880</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>9780310447320</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>9780310447368</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>9780310447528</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>9780310447542</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>9780310447702</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>9780310448334</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>9780310448624</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>9780310448655</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>9780310448839</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>9780310448976</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>9780310448983</v>
       </c>
@@ -3603,7 +3603,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>9780310449027</v>
       </c>
@@ -3635,7 +3635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>9780310449126</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>9780310449133</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>9780310449157</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>9780310449164</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>9780310449188</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>9780310449195</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>9780310449201</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>9780310449430</v>
       </c>
@@ -3891,7 +3891,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>9780310449645</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>9780310449713</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>9780310450023</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>9780310450382</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>9780310450399</v>
       </c>
@@ -4083,7 +4083,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>9780310450573</v>
       </c>
@@ -4115,7 +4115,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>9780310450788</v>
       </c>
@@ -4147,7 +4147,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>9780310452195</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>9780310452201</v>
       </c>
@@ -4211,7 +4211,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>9780310452256</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>9780310452300</v>
       </c>
@@ -4275,7 +4275,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>9780310453093</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>9780310453109</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>9780310453444</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>9780310453505</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>9780310453727</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>9780310454267</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>9780310454465</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>9780310454847</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>9780310454915</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>9780310454960</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>9780310454984</v>
       </c>
@@ -4627,7 +4627,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>9780310455028</v>
       </c>
@@ -4659,7 +4659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>9780310455080</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>9780310455097</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>9780310455196</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>9780310455493</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>9780310455851</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>9780310455882</v>
       </c>
@@ -4851,7 +4851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>9780310455905</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>9780310456292</v>
       </c>
@@ -4947,7 +4947,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>9780310456513</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>9780310456575</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>9780310456674</v>
       </c>
@@ -5043,7 +5043,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>9780310457534</v>
       </c>
@@ -5075,7 +5075,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>9780310457541</v>
       </c>
@@ -5107,7 +5107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>9780310458197</v>
       </c>
@@ -5139,7 +5139,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>9780310458685</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>9780310458746</v>
       </c>
@@ -5203,7 +5203,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>9780310458951</v>
       </c>
@@ -5235,7 +5235,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>9780310459002</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>9780310459040</v>
       </c>
@@ -5299,7 +5299,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>9780310459057</v>
       </c>
@@ -5331,7 +5331,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>9780310459187</v>
       </c>
@@ -5363,7 +5363,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>9780310459231</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="98" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>9780310459347</v>
       </c>
@@ -5427,7 +5427,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>9780310459354</v>
       </c>
@@ -5459,7 +5459,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>9780310459408</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>9780310459545</v>
       </c>
@@ -5523,7 +5523,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>9780310459552</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>9780310459682</v>
       </c>
@@ -5587,7 +5587,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>9780310459743</v>
       </c>
@@ -5619,7 +5619,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>9780310459828</v>
       </c>
@@ -5651,7 +5651,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>9780310459835</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>9780310460138</v>
       </c>
@@ -5715,7 +5715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>9780310460633</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="109" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>9780310460640</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>9780310460695</v>
       </c>
@@ -5811,7 +5811,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>9780310460718</v>
       </c>
@@ -5843,7 +5843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>9780310460886</v>
       </c>
@@ -5875,7 +5875,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>9780310461128</v>
       </c>
@@ -5907,7 +5907,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>9780310461203</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>9780310461562</v>
       </c>
@@ -5971,7 +5971,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>9780310461579</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>9780310461609</v>
       </c>
@@ -6035,7 +6035,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>9780310461807</v>
       </c>
@@ -6067,7 +6067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>9780310461821</v>
       </c>
@@ -6099,7 +6099,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>9780310461869</v>
       </c>
@@ -6131,7 +6131,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>9780310461876</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>9780310461890</v>
       </c>
@@ -6195,7 +6195,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>9780310462033</v>
       </c>
@@ -6227,7 +6227,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>9780310462125</v>
       </c>
@@ -6259,7 +6259,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>9780310462200</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>9780310462477</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>9780310462484</v>
       </c>
@@ -6355,7 +6355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>9780310462491</v>
       </c>
@@ -6387,7 +6387,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>9780310462859</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>9780310462880</v>
       </c>
@@ -6451,7 +6451,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>9780310462897</v>
       </c>
@@ -6483,7 +6483,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>9780310462927</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="133" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>9780310462996</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="134" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>9780310463146</v>
       </c>
@@ -6579,7 +6579,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>9780310463474</v>
       </c>
@@ -6611,7 +6611,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>9780310463481</v>
       </c>
@@ -6643,7 +6643,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="137" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>9780310463498</v>
       </c>
@@ -6675,7 +6675,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>9780310463801</v>
       </c>
@@ -6707,7 +6707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>9780310463863</v>
       </c>
@@ -6739,7 +6739,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>9780310463900</v>
       </c>
@@ -6771,7 +6771,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>9780310463931</v>
       </c>
@@ -6803,7 +6803,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>9780310463986</v>
       </c>
@@ -6835,7 +6835,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>9780310464006</v>
       </c>
@@ -6867,7 +6867,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>9780310464044</v>
       </c>
@@ -6899,7 +6899,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="145" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>9780310464181</v>
       </c>
@@ -6931,7 +6931,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>9780310464457</v>
       </c>
@@ -6963,7 +6963,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="147" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>9780310465065</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>9780310465096</v>
       </c>
@@ -7027,7 +7027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>9780310465102</v>
       </c>
@@ -7059,7 +7059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>9780310465157</v>
       </c>
@@ -7091,7 +7091,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>9780310465249</v>
       </c>
@@ -7123,7 +7123,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>9780310465256</v>
       </c>
@@ -7155,7 +7155,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="153" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>9780310465263</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="154" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>9780310465270</v>
       </c>
@@ -7219,7 +7219,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>9780310465287</v>
       </c>
@@ -7251,7 +7251,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>9780310465294</v>
       </c>
@@ -7283,7 +7283,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>9780310465300</v>
       </c>
@@ -7315,7 +7315,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>9780310465331</v>
       </c>
@@ -7347,7 +7347,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>9780310465348</v>
       </c>
@@ -7379,7 +7379,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>9780310465508</v>
       </c>
@@ -7411,7 +7411,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>9780310465553</v>
       </c>
@@ -7443,7 +7443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>9780310465584</v>
       </c>
@@ -7475,7 +7475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>9780310465799</v>
       </c>
@@ -7507,7 +7507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="164" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>9780310465805</v>
       </c>
@@ -7539,7 +7539,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="165" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>9780310465812</v>
       </c>
@@ -7571,7 +7571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="166" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>9780310465836</v>
       </c>
@@ -7603,7 +7603,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="167" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>9780310465867</v>
       </c>
@@ -7731,7 +7731,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="171" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>9780310466482</v>
       </c>
@@ -7795,7 +7795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="173" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>9780310467571</v>
       </c>
@@ -7827,7 +7827,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="174" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>9780310621829</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="177" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>9780310727484</v>
       </c>
@@ -8051,7 +8051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="181" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>9780310763154</v>
       </c>
@@ -8083,7 +8083,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="182" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>9780310763246</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="183" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>9780310763253</v>
       </c>
@@ -8147,7 +8147,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="184" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>9780310763536</v>
       </c>
@@ -8211,7 +8211,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="186" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>9780310764267</v>
       </c>
@@ -8243,7 +8243,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="187" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>9780310765776</v>
       </c>
@@ -8275,7 +8275,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="188" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>9780310765837</v>
       </c>
@@ -8403,7 +8403,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="192" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>9780529106537</v>
       </c>
@@ -8595,7 +8595,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="198" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>9780718074463</v>
       </c>
@@ -8627,7 +8627,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="199" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>9780718074791</v>
       </c>
@@ -8659,7 +8659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="200" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>9780718074876</v>
       </c>
@@ -8691,7 +8691,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="201" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>9780718075163</v>
       </c>
@@ -8723,7 +8723,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="202" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A202">
         <v>9780718075262</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="203" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A203">
         <v>9780718075279</v>
       </c>
@@ -8787,7 +8787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="204" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A204">
         <v>9780718075514</v>
       </c>
@@ -8819,7 +8819,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="205" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A205">
         <v>9780718075521</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="206" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A206">
         <v>9780718075538</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="207" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A207">
         <v>9780718075583</v>
       </c>
@@ -8915,7 +8915,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="208" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A208">
         <v>9780718075606</v>
       </c>
@@ -8947,7 +8947,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="209" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>9780718075651</v>
       </c>
@@ -8979,7 +8979,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="210" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>9780718079154</v>
       </c>
@@ -9011,7 +9011,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="211" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>9780718079758</v>
       </c>
@@ -9043,7 +9043,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="212" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>9780718079772</v>
       </c>
@@ -9075,7 +9075,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="213" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A213">
         <v>9780718079789</v>
       </c>
@@ -9107,7 +9107,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="214" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>9780718079871</v>
       </c>
@@ -9139,7 +9139,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="215" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A215">
         <v>9780718079895</v>
       </c>
@@ -9171,7 +9171,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="216" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A216">
         <v>9780718086770</v>
       </c>
@@ -9203,7 +9203,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="217" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A217">
         <v>9780718091736</v>
       </c>
@@ -9235,7 +9235,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="218" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A218">
         <v>9780718095444</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="219" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A219">
         <v>9780718095567</v>
       </c>
@@ -9299,7 +9299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="220" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A220">
         <v>9780718095635</v>
       </c>
@@ -9331,7 +9331,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="221" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A221">
         <v>9780718096014</v>
       </c>
@@ -9363,7 +9363,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="222" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A222">
         <v>9780718096793</v>
       </c>
@@ -9395,7 +9395,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A223">
         <v>9780718097264</v>
       </c>
@@ -9427,7 +9427,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="224" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A224">
         <v>9780718097295</v>
       </c>
@@ -9459,7 +9459,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="225" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A225">
         <v>9780718097301</v>
       </c>
@@ -9491,7 +9491,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="226" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A226">
         <v>9780718097325</v>
       </c>
@@ -9523,7 +9523,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="227" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A227">
         <v>9780718097561</v>
       </c>
@@ -9555,7 +9555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="228" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A228">
         <v>9780718097578</v>
       </c>
@@ -9587,7 +9587,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="229" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A229">
         <v>9780718097585</v>
       </c>
@@ -9619,7 +9619,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="230" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>9780718097790</v>
       </c>
@@ -9651,7 +9651,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="231" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A231">
         <v>9780718097820</v>
       </c>
@@ -9683,7 +9683,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="232" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A232">
         <v>9780718097905</v>
       </c>
@@ -9715,7 +9715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="233" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A233">
         <v>9780718097936</v>
       </c>
@@ -9747,7 +9747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="234" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A234">
         <v>9780718097943</v>
       </c>
@@ -9779,7 +9779,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="235" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A235">
         <v>9780718098001</v>
       </c>
@@ -9811,7 +9811,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="236" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A236">
         <v>9780718098025</v>
       </c>
@@ -9843,7 +9843,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="237" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A237">
         <v>9780718098056</v>
       </c>
@@ -9875,7 +9875,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="238" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A238">
         <v>9780718098063</v>
       </c>
@@ -9907,7 +9907,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="239" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A239">
         <v>9780718098070</v>
       </c>
@@ -9939,7 +9939,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="240" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A240">
         <v>9780718098087</v>
       </c>
@@ -9971,7 +9971,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="241" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A241">
         <v>9780718098193</v>
       </c>
@@ -10003,7 +10003,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="242" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A242">
         <v>9780718098216</v>
       </c>
@@ -10035,7 +10035,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="243" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A243">
         <v>9780718098230</v>
       </c>
@@ -10067,7 +10067,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="244" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A244">
         <v>9780718098247</v>
       </c>
@@ -10099,7 +10099,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="245" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A245">
         <v>9780718098254</v>
       </c>
@@ -10131,7 +10131,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="246" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>9780785212379</v>
       </c>
@@ -10163,7 +10163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="247" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A247">
         <v>9780785215158</v>
       </c>
@@ -10195,7 +10195,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="248" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A248">
         <v>9780785215356</v>
       </c>
@@ -10227,7 +10227,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="249" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A249">
         <v>9780785215363</v>
       </c>
@@ -10259,7 +10259,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="250" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A250">
         <v>9780785215394</v>
       </c>
@@ -10291,7 +10291,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="251" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A251">
         <v>9780785215417</v>
       </c>
@@ -10323,7 +10323,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="252" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A252">
         <v>9780785215462</v>
       </c>
@@ -10355,7 +10355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="253" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A253">
         <v>9780785215493</v>
       </c>
@@ -10387,7 +10387,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="254" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A254">
         <v>9780785215509</v>
       </c>
@@ -10419,7 +10419,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="255" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A255">
         <v>9780785215523</v>
       </c>
@@ -10451,7 +10451,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="256" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A256">
         <v>9780785215547</v>
       </c>
@@ -10483,7 +10483,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="257" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A257">
         <v>9780785215554</v>
       </c>
@@ -10515,7 +10515,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="258" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A258">
         <v>9780785215615</v>
       </c>
@@ -10547,7 +10547,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="259" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A259">
         <v>9780785215646</v>
       </c>
@@ -10579,7 +10579,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="260" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A260">
         <v>9780785215653</v>
       </c>
@@ -10611,7 +10611,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="261" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A261">
         <v>9780785215677</v>
       </c>
@@ -10643,7 +10643,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="262" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>9780785215684</v>
       </c>
@@ -10675,7 +10675,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="263" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A263">
         <v>9780785215707</v>
       </c>
@@ -10707,7 +10707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="264" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A264">
         <v>9780785215714</v>
       </c>
@@ -10739,7 +10739,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="265" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A265">
         <v>9780785215738</v>
       </c>
@@ -10771,7 +10771,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="266" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A266">
         <v>9780785215820</v>
       </c>
@@ -10803,7 +10803,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="267" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A267">
         <v>9780785215936</v>
       </c>
@@ -10835,7 +10835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="268" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A268">
         <v>9780785216711</v>
       </c>
@@ -10867,7 +10867,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="269" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A269">
         <v>9780785217039</v>
       </c>
@@ -10899,7 +10899,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="270" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A270">
         <v>9780785217664</v>
       </c>
@@ -10931,7 +10931,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="271" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A271">
         <v>9780785217701</v>
       </c>
@@ -10963,7 +10963,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="272" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A272">
         <v>9780785217732</v>
       </c>
@@ -10995,7 +10995,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="273" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A273">
         <v>9780785218005</v>
       </c>
@@ -11027,7 +11027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="274" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A274">
         <v>9780785218159</v>
       </c>
@@ -11059,7 +11059,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="275" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A275">
         <v>9780785218623</v>
       </c>
@@ -11091,7 +11091,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="276" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A276">
         <v>9780785220480</v>
       </c>
@@ -11123,7 +11123,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A277">
         <v>9780785220589</v>
       </c>
@@ -11155,7 +11155,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>9780785220671</v>
       </c>
@@ -11187,7 +11187,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="279" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A279">
         <v>9780785220688</v>
       </c>
@@ -11219,7 +11219,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="280" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A280">
         <v>9780785222439</v>
       </c>
@@ -11251,7 +11251,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="281" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A281">
         <v>9780785222484</v>
       </c>
@@ -11283,7 +11283,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="282" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A282">
         <v>9780785222941</v>
       </c>
@@ -11315,7 +11315,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="283" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A283">
         <v>9780785223085</v>
       </c>
@@ -11347,7 +11347,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="284" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A284">
         <v>9780785223092</v>
       </c>
@@ -11379,7 +11379,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="285" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A285">
         <v>9780785223108</v>
       </c>
@@ -11411,7 +11411,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="286" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A286">
         <v>9780785225577</v>
       </c>
@@ -11443,7 +11443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="287" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A287">
         <v>9780785225607</v>
       </c>
@@ -11475,7 +11475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="288" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A288">
         <v>9780785225874</v>
       </c>
@@ -11507,7 +11507,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="289" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A289">
         <v>9780785225904</v>
       </c>
@@ -11539,7 +11539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="290" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A290">
         <v>9780785225935</v>
       </c>
@@ -11571,7 +11571,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="291" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A291">
         <v>9780785225966</v>
       </c>
@@ -11603,7 +11603,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="292" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A292">
         <v>9780785225980</v>
       </c>
@@ -11635,7 +11635,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="293" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A293">
         <v>9780785227540</v>
       </c>
@@ -11667,7 +11667,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="294" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A294">
         <v>9780785227557</v>
       </c>
@@ -11699,7 +11699,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="295" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A295">
         <v>9780785230236</v>
       </c>
@@ -11731,7 +11731,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="296" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A296">
         <v>9780785230311</v>
       </c>
@@ -11763,7 +11763,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A297">
         <v>9780785230328</v>
       </c>
@@ -11795,7 +11795,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A298">
         <v>9780785230335</v>
       </c>
@@ -11827,7 +11827,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="299" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A299">
         <v>9780785230342</v>
       </c>
@@ -11859,7 +11859,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="300" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A300">
         <v>9780785231660</v>
       </c>
@@ -11891,7 +11891,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="301" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A301">
         <v>9780785231721</v>
       </c>
@@ -11923,7 +11923,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="302" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A302">
         <v>9780785233268</v>
       </c>
@@ -11955,7 +11955,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="303" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A303">
         <v>9780785235507</v>
       </c>
@@ -11987,7 +11987,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="304" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A304">
         <v>9780785235514</v>
       </c>
@@ -12019,7 +12019,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A305">
         <v>9780785235521</v>
       </c>
@@ -12051,7 +12051,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="306" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A306">
         <v>9780785235644</v>
       </c>
@@ -12083,7 +12083,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="307" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A307">
         <v>9780785235651</v>
       </c>
@@ -12275,7 +12275,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="313" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A313">
         <v>9780785237594</v>
       </c>
@@ -12307,7 +12307,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="314" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A314">
         <v>9780785237600</v>
       </c>
@@ -12339,7 +12339,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="315" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A315">
         <v>9780785237884</v>
       </c>
@@ -12371,7 +12371,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="316" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A316">
         <v>9780785238010</v>
       </c>
@@ -12403,7 +12403,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="317" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A317">
         <v>9780785238072</v>
       </c>
@@ -12435,7 +12435,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="318" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A318">
         <v>9780785238287</v>
       </c>
@@ -12467,7 +12467,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="319" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A319">
         <v>9780785238416</v>
       </c>
@@ -12499,7 +12499,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="320" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A320">
         <v>9780785239062</v>
       </c>
@@ -12531,7 +12531,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="321" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A321">
         <v>9780785239246</v>
       </c>
@@ -12563,7 +12563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="322" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A322">
         <v>9780785239277</v>
       </c>
@@ -12595,7 +12595,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="323" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A323">
         <v>9780785239314</v>
       </c>
@@ -12627,7 +12627,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="324" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A324">
         <v>9780785239581</v>
       </c>
@@ -12659,7 +12659,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="325" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A325">
         <v>9780785241812</v>
       </c>
@@ -12691,7 +12691,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="326" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A326">
         <v>9780785241898</v>
       </c>
@@ -12723,7 +12723,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="327" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A327">
         <v>9780785241911</v>
       </c>
@@ -12755,7 +12755,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="328" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A328">
         <v>9780785241928</v>
       </c>
@@ -12787,7 +12787,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="329" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A329">
         <v>9780785241942</v>
       </c>
@@ -12819,7 +12819,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="330" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A330">
         <v>9780785241997</v>
       </c>
@@ -12851,7 +12851,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="331" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A331">
         <v>9780785242185</v>
       </c>
@@ -12883,7 +12883,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="332" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A332">
         <v>9780785246664</v>
       </c>
@@ -12915,7 +12915,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="333" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A333">
         <v>9780785246688</v>
       </c>
@@ -12979,7 +12979,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="335" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A335">
         <v>9780785248637</v>
       </c>
@@ -13011,7 +13011,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="336" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A336">
         <v>9780785248651</v>
       </c>
@@ -13043,7 +13043,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="337" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A337">
         <v>9780785248811</v>
       </c>
@@ -13075,7 +13075,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="338" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A338">
         <v>9780785250746</v>
       </c>
@@ -13107,7 +13107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="339" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A339">
         <v>9780785250838</v>
       </c>
@@ -13139,7 +13139,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="340" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A340">
         <v>9780785250869</v>
       </c>
@@ -13171,7 +13171,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="341" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A341">
         <v>9780785253235</v>
       </c>
@@ -13203,7 +13203,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="342" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A342">
         <v>9780785253334</v>
       </c>
@@ -13235,7 +13235,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="343" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A343">
         <v>9780785253358</v>
       </c>
@@ -13267,7 +13267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="344" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A344">
         <v>9780785253365</v>
       </c>
@@ -13299,7 +13299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="345" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A345">
         <v>9780785253396</v>
       </c>
@@ -13331,7 +13331,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="346" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A346">
         <v>9780785253402</v>
       </c>
@@ -13363,7 +13363,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="347" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A347">
         <v>9780785253488</v>
       </c>
@@ -13395,7 +13395,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="348" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A348">
         <v>9780785255574</v>
       </c>
@@ -13427,7 +13427,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="349" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A349">
         <v>9780785255598</v>
       </c>
@@ -13459,7 +13459,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="350" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A350">
         <v>9780785259497</v>
       </c>
@@ -13491,7 +13491,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="351" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A351">
         <v>9780785261599</v>
       </c>
@@ -13619,7 +13619,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="355" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A355">
         <v>9780785289074</v>
       </c>
@@ -13651,7 +13651,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="356" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A356">
         <v>9780785290148</v>
       </c>
@@ -13683,7 +13683,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="357" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A357">
         <v>9780785290155</v>
       </c>
@@ -13715,7 +13715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="358" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A358">
         <v>9780785290162</v>
       </c>
@@ -13747,7 +13747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="359" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A359">
         <v>9780785291107</v>
       </c>
@@ -13779,7 +13779,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="360" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A360">
         <v>9780785291121</v>
       </c>
@@ -13811,7 +13811,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="361" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A361">
         <v>9780785291169</v>
       </c>
@@ -13843,7 +13843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="362" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A362">
         <v>9780785291176</v>
       </c>
@@ -13875,7 +13875,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="363" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A363">
         <v>9780785291183</v>
       </c>
@@ -13907,7 +13907,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="364" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A364">
         <v>9780785291190</v>
       </c>
@@ -13939,7 +13939,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="365" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A365">
         <v>9780785291206</v>
       </c>
@@ -13971,7 +13971,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="366" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A366">
         <v>9780785291244</v>
       </c>
@@ -14003,7 +14003,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A367">
         <v>9780785291442</v>
       </c>
@@ -14035,7 +14035,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A368">
         <v>9780785291480</v>
       </c>
@@ -14067,7 +14067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A369">
         <v>9780785291497</v>
       </c>
@@ -14099,7 +14099,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="370" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A370">
         <v>9780785291503</v>
       </c>
@@ -14131,7 +14131,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="371" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A371">
         <v>9780785291589</v>
       </c>
@@ -14163,7 +14163,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A372">
         <v>9780785292760</v>
       </c>
@@ -14195,7 +14195,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="373" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A373">
         <v>9780785292814</v>
       </c>
@@ -14227,7 +14227,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="374" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A374">
         <v>9780785292821</v>
       </c>
@@ -14259,7 +14259,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="375" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A375">
         <v>9780785292890</v>
       </c>
@@ -14291,7 +14291,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="376" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A376">
         <v>9780785292906</v>
       </c>
@@ -14323,7 +14323,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="377" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A377">
         <v>9780785292951</v>
       </c>
@@ -14355,7 +14355,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="378" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A378">
         <v>9780785293231</v>
       </c>
@@ -14387,7 +14387,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="379" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A379">
         <v>9780785293248</v>
       </c>
@@ -14419,7 +14419,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="380" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A380">
         <v>9780785294504</v>
       </c>
@@ -14451,7 +14451,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="381" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A381">
         <v>9780785294559</v>
       </c>
@@ -14483,7 +14483,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="382" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A382">
         <v>9780785294566</v>
       </c>
@@ -14515,7 +14515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="383" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A383">
         <v>9780785294580</v>
       </c>
@@ -14547,7 +14547,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="384" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A384">
         <v>9780785294894</v>
       </c>
@@ -14579,7 +14579,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="385" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A385">
         <v>9780785294948</v>
       </c>
@@ -14803,7 +14803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="392" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A392">
         <v>9780785296287</v>
       </c>
@@ -14835,7 +14835,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="393" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A393">
         <v>9780785296294</v>
       </c>
@@ -14867,7 +14867,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="394" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A394">
         <v>9780785296300</v>
       </c>
@@ -14899,7 +14899,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="395" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A395">
         <v>9780785296317</v>
       </c>
@@ -14931,7 +14931,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="396" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A396">
         <v>9780785296324</v>
       </c>
@@ -14963,7 +14963,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="397" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A397">
         <v>9780785296331</v>
       </c>
@@ -14995,7 +14995,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="398" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A398">
         <v>9780785297390</v>
       </c>
@@ -15027,7 +15027,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="399" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A399">
         <v>9780785297819</v>
       </c>
@@ -15059,7 +15059,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="400" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A400">
         <v>9780829771169</v>
       </c>
@@ -15219,7 +15219,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="405" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A405">
         <v>9781400328772</v>
       </c>
@@ -15251,7 +15251,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="406" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A406">
         <v>9781400330829</v>
       </c>
@@ -15283,7 +15283,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="407" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A407">
         <v>9781400330867</v>
       </c>
@@ -15315,7 +15315,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="408" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A408">
         <v>9781400331123</v>
       </c>
@@ -15347,7 +15347,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="409" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A409">
         <v>9781400331178</v>
       </c>
@@ -15379,7 +15379,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="410" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A410">
         <v>9781400331437</v>
       </c>
@@ -15411,7 +15411,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="411" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A411">
         <v>9781400331765</v>
       </c>
@@ -15443,7 +15443,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="412" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A412">
         <v>9781400332038</v>
       </c>
@@ -15475,7 +15475,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="413" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A413">
         <v>9781400332083</v>
       </c>
@@ -15507,7 +15507,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="414" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="414" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A414">
         <v>9781400332274</v>
       </c>
@@ -15539,7 +15539,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="415" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A415">
         <v>9781400332311</v>
       </c>
@@ -15571,7 +15571,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="416" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A416">
         <v>9781400332403</v>
       </c>
@@ -15603,7 +15603,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="417" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A417">
         <v>9781400332496</v>
       </c>
@@ -15635,7 +15635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="418" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="418" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A418">
         <v>9781400332571</v>
       </c>
@@ -15667,7 +15667,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="419" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="419" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A419">
         <v>9781400333028</v>
       </c>
@@ -15699,7 +15699,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="420" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="420" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A420">
         <v>9781400333035</v>
       </c>
@@ -15731,7 +15731,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="421" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="421" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A421">
         <v>9781400333097</v>
       </c>
@@ -15763,7 +15763,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="422" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="422" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A422">
         <v>9781400333110</v>
       </c>
@@ -15795,7 +15795,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="423" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="423" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A423">
         <v>9781400333127</v>
       </c>
@@ -15827,7 +15827,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="424" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="424" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A424">
         <v>9781400333141</v>
       </c>
@@ -15859,7 +15859,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="425" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="425" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A425">
         <v>9781400333158</v>
       </c>
@@ -15891,7 +15891,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="426" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="426" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A426">
         <v>9781400333165</v>
       </c>
@@ -15923,7 +15923,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="427" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="427" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A427">
         <v>9781400333370</v>
       </c>
@@ -15987,7 +15987,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="429" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="429" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A429">
         <v>9781400333479</v>
       </c>
@@ -16083,7 +16083,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="432" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="432" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A432">
         <v>9781400335350</v>
       </c>
@@ -16115,7 +16115,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="433" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="433" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A433">
         <v>9781400335367</v>
       </c>
@@ -16147,7 +16147,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="434" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="434" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A434">
         <v>9781400335398</v>
       </c>
@@ -16211,7 +16211,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="436" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="436" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A436">
         <v>9781400335459</v>
       </c>
@@ -16275,7 +16275,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="438" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A438">
         <v>9781400336012</v>
       </c>
@@ -16307,7 +16307,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="439" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="439" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A439">
         <v>9781400336746</v>
       </c>
@@ -16339,7 +16339,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="440" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A440">
         <v>9781400337545</v>
       </c>
@@ -16371,7 +16371,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="441" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="441" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A441">
         <v>9781400337569</v>
       </c>
@@ -16403,7 +16403,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="442" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="442" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A442">
         <v>9781400337941</v>
       </c>
@@ -16435,7 +16435,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="443" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="443" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A443">
         <v>9781400338306</v>
       </c>
@@ -16467,7 +16467,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="444" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="444" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A444">
         <v>9781400338337</v>
       </c>
@@ -16499,7 +16499,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="445" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A445">
         <v>9781400338412</v>
       </c>
@@ -16531,7 +16531,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="446" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A446">
         <v>9781400338429</v>
       </c>
@@ -16563,7 +16563,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="447" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A447">
         <v>9781400338436</v>
       </c>
@@ -16627,7 +16627,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="449" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="449" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A449">
         <v>9781400338559</v>
       </c>
@@ -16755,7 +16755,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="453" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="453" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A453">
         <v>9781400339754</v>
       </c>
@@ -16883,7 +16883,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="457" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="457" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A457">
         <v>9781400341887</v>
       </c>
@@ -17011,7 +17011,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="461" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A461">
         <v>9781400344031</v>
       </c>
@@ -17043,7 +17043,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="462" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="462" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A462">
         <v>9781400344079</v>
       </c>
@@ -17075,7 +17075,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="463" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="463" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A463">
         <v>9781400344086</v>
       </c>
@@ -17107,7 +17107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="464" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="464" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A464">
         <v>9781400344116</v>
       </c>
@@ -17139,7 +17139,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="465" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="465" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A465">
         <v>9781400344154</v>
       </c>
@@ -17171,7 +17171,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="466" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="466" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A466">
         <v>9781400344192</v>
       </c>
@@ -17203,7 +17203,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="467" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="467" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A467">
         <v>9781400344239</v>
       </c>
@@ -17235,7 +17235,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="468" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="468" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A468">
         <v>9781400344352</v>
       </c>
@@ -17267,7 +17267,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="469" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="469" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A469">
         <v>9781400345403</v>
       </c>
@@ -17299,7 +17299,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="470" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="470" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A470">
         <v>9781400345410</v>
       </c>
@@ -17363,7 +17363,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="472" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="472" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A472">
         <v>9781400345489</v>
       </c>
@@ -17395,7 +17395,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="473" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="473" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A473">
         <v>9781400345496</v>
       </c>
@@ -17427,7 +17427,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="474" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="474" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A474">
         <v>9781400346325</v>
       </c>
@@ -17459,7 +17459,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="475" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="475" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A475">
         <v>9781400346332</v>
       </c>
@@ -17491,7 +17491,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="476" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="476" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A476">
         <v>9781400349081</v>
       </c>
@@ -17523,7 +17523,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="477" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="477" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A477">
         <v>9781400349432</v>
       </c>
@@ -17555,7 +17555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="478" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="478" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A478">
         <v>9781400349715</v>
       </c>
@@ -17619,7 +17619,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="480" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="480" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A480">
         <v>9781400350582</v>
       </c>
@@ -17715,7 +17715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="483" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="483" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A483">
         <v>9781401679538</v>
       </c>
@@ -17747,7 +17747,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="484" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="484" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A484">
         <v>9781401679569</v>
       </c>
@@ -17779,7 +17779,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="485" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="485" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A485">
         <v>9781401679590</v>
       </c>
@@ -17811,7 +17811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="486" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="486" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A486">
         <v>9781401680367</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="497" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="497" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A497">
         <v>9781496447227</v>
       </c>
@@ -18195,7 +18195,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="498" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="498" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A498">
         <v>9781496447234</v>
       </c>
@@ -18227,7 +18227,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="499" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="499" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A499">
         <v>9781496447258</v>
       </c>
@@ -18291,7 +18291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="501" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="501" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A501">
         <v>9781496472137</v>
       </c>
@@ -18355,7 +18355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="503" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="503" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A503">
         <v>9781623371449</v>
       </c>
@@ -18387,7 +18387,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="504" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="504" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A504">
         <v>9781683073697</v>
       </c>
@@ -18419,7 +18419,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="505" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="505" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A505">
         <v>9780310448945</v>
       </c>
@@ -18451,7 +18451,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="506" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="506" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A506">
         <v>9780310459606</v>
       </c>
@@ -18483,7 +18483,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="507" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="507" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A507">
         <v>9780310459699</v>
       </c>
@@ -18515,7 +18515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="508" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="508" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A508">
         <v>9780310460251</v>
       </c>
@@ -18547,7 +18547,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="509" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="509" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A509">
         <v>9780310460398</v>
       </c>
@@ -18579,7 +18579,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="510" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="510" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A510">
         <v>9780310460817</v>
       </c>
@@ -18611,7 +18611,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="511" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="511" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A511">
         <v>9780785226642</v>
       </c>
@@ -18643,7 +18643,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="512" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="512" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A512">
         <v>9780785241867</v>
       </c>
@@ -18675,7 +18675,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="513" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="513" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A513">
         <v>9780785263081</v>
       </c>
@@ -18707,7 +18707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="514" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="514" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A514">
         <v>9780785296089</v>
       </c>
@@ -18739,7 +18739,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="515" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="515" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A515">
         <v>9780310461562</v>
       </c>
@@ -18771,7 +18771,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="516" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="516" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A516">
         <v>9780785291169</v>
       </c>
@@ -18803,7 +18803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="517" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="517" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A517">
         <v>9781400330010</v>
       </c>
@@ -18867,7 +18867,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="519" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="519" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A519">
         <v>9780310452966</v>
       </c>
@@ -18899,7 +18899,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="520" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="520" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A520">
         <v>9780310463443</v>
       </c>
@@ -18931,7 +18931,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="521" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="521" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A521">
         <v>9780718097301</v>
       </c>
@@ -18963,7 +18963,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="522" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="522" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A522">
         <v>9780310446460</v>
       </c>
@@ -18995,7 +18995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="523" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="523" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A523">
         <v>9780310460572</v>
       </c>
@@ -19027,7 +19027,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="524" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="524" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A524">
         <v>9780718091736</v>
       </c>
@@ -19059,7 +19059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="525" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="525" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A525">
         <v>9780310445890</v>
       </c>
@@ -19091,7 +19091,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="526" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="526" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A526">
         <v>9780310448945</v>
       </c>
@@ -19123,7 +19123,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="527" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="527" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A527">
         <v>9780785295709</v>
       </c>
@@ -19155,7 +19155,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="528" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="528" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A528">
         <v>9781404110090</v>
       </c>
@@ -19187,7 +19187,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="529" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="529" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A529">
         <v>9780310447146</v>
       </c>
@@ -19219,7 +19219,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="530" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="530" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A530">
         <v>9780310450559</v>
       </c>
@@ -19251,7 +19251,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="531" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="531" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A531">
         <v>9781400330010</v>
       </c>
@@ -19283,7 +19283,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="532" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="532" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A532">
         <v>9780785290339</v>
       </c>
@@ -19315,7 +19315,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="533" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="533" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A533">
         <v>9780310764076</v>
       </c>
@@ -19347,7 +19347,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="534" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="534" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A534">
         <v>9781400336012</v>
       </c>
@@ -19379,7 +19379,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="535" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="535" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A535">
         <v>9780785295990</v>
       </c>
@@ -19411,7 +19411,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="536" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="536" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A536">
         <v>9781418542290</v>
       </c>
@@ -19443,7 +19443,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="537" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="537" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A537">
         <v>9780310445890</v>
       </c>
@@ -19475,7 +19475,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="538" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="538" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A538">
         <v>9780310448945</v>
       </c>
@@ -19507,7 +19507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="539" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="539" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A539">
         <v>9780785263081</v>
       </c>
@@ -19539,7 +19539,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="540" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="540" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A540">
         <v>9780785250869</v>
       </c>
@@ -19571,7 +19571,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="541" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="541" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A541">
         <v>9780310459606</v>
       </c>
@@ -19603,7 +19603,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="542" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="542" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A542">
         <v>9781404110113</v>
       </c>
@@ -19635,7 +19635,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="543" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="543" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A543">
         <v>9780785250838</v>
       </c>
@@ -19667,7 +19667,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="544" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="544" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A544">
         <v>9781400333059</v>
       </c>
@@ -19699,7 +19699,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="545" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="545" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A545">
         <v>9780785250845</v>
       </c>
@@ -19731,7 +19731,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="546" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="546" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A546">
         <v>9780310763536</v>
       </c>
@@ -19763,7 +19763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="547" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="547" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A547">
         <v>9781400333165</v>
       </c>
@@ -19795,7 +19795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="548" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="548" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A548">
         <v>9781400333141</v>
       </c>
@@ -19827,7 +19827,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="549" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="549" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A549">
         <v>9781400333127</v>
       </c>
@@ -19859,7 +19859,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="550" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="550" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A550">
         <v>9780785296324</v>
       </c>
@@ -19891,7 +19891,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="551" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="551" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A551">
         <v>9780785296331</v>
       </c>
@@ -19923,7 +19923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="552" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="552" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A552">
         <v>9780785293255</v>
       </c>
@@ -19955,7 +19955,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="553" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="553" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A553">
         <v>9780785293231</v>
       </c>
@@ -19987,7 +19987,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="554" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="554" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A554">
         <v>9780785296317</v>
       </c>
@@ -20019,7 +20019,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="555" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="555" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A555">
         <v>9780785296287</v>
       </c>
@@ -20051,7 +20051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="556" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="556" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A556">
         <v>9780785296300</v>
       </c>
@@ -20083,7 +20083,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="557" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="557" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A557">
         <v>9780785296294</v>
       </c>
@@ -20115,7 +20115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="558" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="558" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A558">
         <v>9780785293248</v>
       </c>
@@ -20147,7 +20147,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="559" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="559" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A559">
         <v>9781400338337</v>
       </c>
@@ -20179,7 +20179,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="560" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="560" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A560">
         <v>9780785294955</v>
       </c>
@@ -20211,7 +20211,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="561" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="561" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A561">
         <v>9780718042523</v>
       </c>
@@ -20243,7 +20243,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="562" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="562" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A562">
         <v>9780785227922</v>
       </c>
@@ -20275,7 +20275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="563" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="563" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A563">
         <v>9780785241850</v>
       </c>
@@ -20307,7 +20307,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="564" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="564" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A564">
         <v>9780310462897</v>
       </c>
@@ -20339,7 +20339,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="565" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="565" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A565">
         <v>9780785242529</v>
       </c>
@@ -20371,7 +20371,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="566" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="566" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A566">
         <v>9780785253389</v>
       </c>
@@ -20403,7 +20403,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="567" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="567" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A567">
         <v>9780310462880</v>
       </c>
@@ -20467,7 +20467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="569" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="569" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A569">
         <v>9780785241935</v>
       </c>
@@ -20499,7 +20499,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="570" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="570" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A570">
         <v>9780785290353</v>
       </c>
@@ -20531,7 +20531,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="571" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="571" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A571">
         <v>9780785291619</v>
       </c>
@@ -20563,7 +20563,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="572" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="572" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A572">
         <v>9781496447227</v>
       </c>
@@ -20595,7 +20595,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="573" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="573" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A573">
         <v>9781496460851</v>
       </c>
@@ -20627,7 +20627,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="574" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="574" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A574">
         <v>9781619707221</v>
       </c>
@@ -20659,7 +20659,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="575" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="575" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A575">
         <v>9781496461452</v>
       </c>
@@ -20691,7 +20691,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="576" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="576" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A576">
         <v>9781496472014</v>
       </c>
@@ -20787,7 +20787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="579" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="579" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A579">
         <v>9781598566277</v>
       </c>
@@ -20819,7 +20819,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="580" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="580" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A580">
         <v>9781496447180</v>
       </c>
@@ -20851,7 +20851,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="581" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="581" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A581">
         <v>9781496461421</v>
       </c>
@@ -20915,7 +20915,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="583" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="583" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A583">
         <v>9780310166344</v>
       </c>
@@ -20947,7 +20947,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="584" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="584" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A584">
         <v>9780310443926</v>
       </c>
@@ -20979,7 +20979,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="585" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="585" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A585">
         <v>9780310419099</v>
       </c>
@@ -21011,7 +21011,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="586" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="586" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A586">
         <v>1433563428</v>
       </c>
@@ -21235,7 +21235,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="593" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="593" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A593">
         <v>9781414302065</v>
       </c>
@@ -21267,7 +21267,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="594" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="594" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A594">
         <v>9780062064929</v>
       </c>
@@ -21299,7 +21299,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="595" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="595" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A595">
         <v>9780310446101</v>
       </c>
@@ -21331,7 +21331,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="596" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="596" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A596">
         <v>9780310446118</v>
       </c>
@@ -21363,7 +21363,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="597" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="597" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A597">
         <v>9780310757047</v>
       </c>
@@ -21395,7 +21395,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="598" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="598" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A598">
         <v>9781400331178</v>
       </c>
@@ -21427,7 +21427,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="599" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="599" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A599">
         <v>9781400333448</v>
       </c>
@@ -21459,7 +21459,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="600" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="600" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A600">
         <v>9781400330867</v>
       </c>
@@ -21491,7 +21491,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="601" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="601" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A601">
         <v>9781400330560</v>
       </c>
@@ -21523,7 +21523,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="602" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="602" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A602">
         <v>9780718097578</v>
       </c>
@@ -21555,7 +21555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="603" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="603" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A603">
         <v>9780718089481</v>
       </c>
@@ -21587,7 +21587,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="604" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="604" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A604">
         <v>9780785294566</v>
       </c>
@@ -21619,7 +21619,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="605" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="605" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A605">
         <v>9780785215448</v>
       </c>
@@ -21651,7 +21651,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="606" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="606" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A606">
         <v>9780785230083</v>
       </c>
@@ -21715,7 +21715,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="608" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="608" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A608">
         <v>9780718098070</v>
       </c>
@@ -21747,7 +21747,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="609" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="609" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A609">
         <v>9780785217664</v>
       </c>
@@ -21779,7 +21779,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="610" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="610" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A610">
         <v>9780785225935</v>
       </c>
@@ -21811,7 +21811,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="611" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="611" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A611">
         <v>9780785225959</v>
       </c>
@@ -21843,7 +21843,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="612" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="612" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A612">
         <v>9780718097981</v>
       </c>
@@ -21875,7 +21875,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="613" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="613" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A613">
         <v>9780785217671</v>
       </c>
@@ -21907,7 +21907,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="614" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="614" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A614">
         <v>9781619705654</v>
       </c>
@@ -21939,7 +21939,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="615" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="615" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A615">
         <v>9780718098230</v>
       </c>
@@ -21971,7 +21971,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="616" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="616" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A616">
         <v>9780785215806</v>
       </c>
@@ -22003,7 +22003,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="617" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="617" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A617">
         <v>9780785224716</v>
       </c>
@@ -22035,7 +22035,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="618" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="618" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A618">
         <v>9780785224730</v>
       </c>
@@ -22067,7 +22067,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="619" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="619" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A619">
         <v>9780785229155</v>
       </c>
@@ -22099,7 +22099,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="620" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="620" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A620">
         <v>9780785229148</v>
       </c>
@@ -22131,7 +22131,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="621" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="621" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A621">
         <v>9780785227649</v>
       </c>
@@ -22163,7 +22163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="622" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="622" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A622">
         <v>9780785227557</v>
       </c>
@@ -22195,7 +22195,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="623" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="623" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A623">
         <v>9780785227526</v>
       </c>
@@ -22227,7 +22227,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="624" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="624" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A624">
         <v>9781400333417</v>
       </c>
@@ -22259,7 +22259,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="625" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="625" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A625">
         <v>9780310458227</v>
       </c>
@@ -22291,7 +22291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="626" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="626" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A626">
         <v>9780718098124</v>
       </c>
@@ -22324,13 +22324,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J626" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="Unknown"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:J626" numberStoredAsText="1"/>

</xml_diff>